<commit_message>
Add QlM 500-Word SSR Draft Editor and Cloud Drive / Faculty Assignment Tracker
</commit_message>
<xml_diff>
--- a/NAAC_Gap_Analysis.xlsx
+++ b/NAAC_Gap_Analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\NAAC – Criterion VI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C641974-10A8-43A1-A119-BAFCEB3984A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C57ED8B1-4757-4B4B-A7B1-98FAD08204FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15600" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="434">
   <si>
     <t>Criterion I — Curricular Aspects (150)</t>
   </si>
@@ -1322,6 +1322,12 @@
   </si>
   <si>
     <t>HR</t>
+  </si>
+  <si>
+    <t>IQAC + Registrar/Administration + All Schools</t>
+  </si>
+  <si>
+    <t>Registrar + IQAC + All Departments</t>
   </si>
 </sst>
 </file>
@@ -1404,7 +1410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1416,6 +1422,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4784,7 +4793,7 @@
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
     </row>
-    <row r="5" spans="1:12" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>338</v>
       </c>
@@ -4803,7 +4812,9 @@
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="6" t="s">
+        <v>432</v>
+      </c>
       <c r="L5" s="2"/>
     </row>
     <row r="6" spans="1:12" ht="38.25" x14ac:dyDescent="0.25">
@@ -4825,7 +4836,9 @@
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
+      <c r="K6" s="6" t="s">
+        <v>433</v>
+      </c>
       <c r="L6" s="2"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>